<commit_message>
Score warm-path via DLA Piper counsel for reachable firms
Applies the #2 warm-path update using DLA Piper (engaged counsel) as the
intro node, contingent on DLA making each intro:
- a16z Bio+Health: STRONG (partner Josh Seidenfeld led an a16z health-AI
  deal at DLA) -> warm-path 4, fit 84 (now tied #1 with Dimension).
- Lux Capital: DLA partner Jonathan Axelrad represents Lux -> warm-path 3,
  fit 80.
- Basis Set: DLA alumni tie to GC Jennifer Lee -> warm-path 3, fit 80.
- Bessemer: named DLA investor-client -> warm-path 3, fit 66.
Notes each row as contingent on DLA; flags that 'Johnny Lam' could not be
verified as a DLA attorney (confirm role). Other firms unchanged (warm 1-2).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AASgEHUdi3Eu3cEx97KCR
</commit_message>
<xml_diff>
--- a/fundraising/coharts-seed-investor-pipeline.xlsx
+++ b/fundraising/coharts-seed-investor-pipeline.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Institutional Seed; target pre-money $25M to $35M (confirm target raise and lead vs participant). Coharts: An Applied AI company, IaaS (never SaaS). Two products: iViz (AI data-analysis workbench, self-serve/PLG) and Foresight (clinical trial simulation, Simulate Success Before Patient One). Traction/proof: Tempus proof-of-concept partnership; Synthon pilot; Foresight validated against real clinical trials both retrospectively and prospectively (including LEAP and TDM1). Angel round closed Aug 2026 on a legacy pre-money SAFE at a $17.5M cap. Most check sizes are Unknown pending PitchBook; personal emails are inferred unless marked Verified. None of these firms are in the HubSpot pipeline (CRM holds pharma/CRO/biotech BD accounts, not investors). CONFLICT FLAGGED: Radical Ventures holds Unlearn.AI (direct Foresight competitor).</t>
+          <t>Institutional Seed; target pre-money $25M to $35M (confirm target raise and lead vs participant). Coharts: An Applied AI company, IaaS (never SaaS). Two products: iViz (AI data-analysis workbench, self-serve/PLG) and Foresight (clinical trial simulation, Simulate Success Before Patient One). Traction/proof: Tempus proof-of-concept partnership; Synthon pilot; Foresight validated against real clinical trials both retrospectively and prospectively (including LEAP and TDM1). Angel round closed Aug 2026 on a legacy pre-money SAFE at a $17.5M cap. Most check sizes are Unknown pending PitchBook; personal emails are inferred unless marked Verified. None of these firms are in the HubSpot pipeline (CRM holds pharma/CRO/biotech BD accounts, not investors). CONFLICT FLAGGED: Radical Ventures holds Unlearn.AI (direct Foresight competitor). WARM-PATH NODE: DLA Piper is engaged counsel (Josh Seidenfeld, ex-Cooley Digital Health chair; confirm 'Johnny Lam' role). DLA warm-path bumps applied to a16z (strong), Bessemer, Lux, Basis Set (plausible), all CONTINGENT on DLA actually making the intro. Other firms remain warm-path 1-2 pending named nodes.</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
-          <t>Route via an a16z bio+health portfolio founder; no named node confirmed.</t>
+          <t>STRONG via DLA Piper (engaged counsel): partner Josh Seidenfeld personally led a16z's Prosper AI health-AI financing at DLA in 2026. Confirm the intro with Seidenfeld.</t>
         </is>
       </c>
       <c r="Q3" s="9" t="n">
@@ -1117,14 +1117,14 @@
         <v>0</v>
       </c>
       <c r="U3" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V3" s="9" t="n">
         <v>5</v>
       </c>
       <c r="W3" s="10">
         <f>MAX(0,ROUND(Q3/5*Weights!$B$3+R3/5*Weights!$B$4+S3/5*Weights!$B$5+T3/5*Weights!$B$6+U3/5*Weights!$B$7+V3/5*Weights!$B$8-L3*Weights!$B$9,0))</f>
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="X3" s="10" t="str">
         <f>IF(W3&gt;=Weights!$B$12,"A",IF(W3&gt;=Weights!$B$13,"B","C"))</f>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="AA3" s="8" t="inlineStr">
         <is>
-          <t>Find a portfolio-founder intro to Yoo (software lens) or Rughani (AI-health).</t>
+          <t>Ask Josh Seidenfeld (DLA Piper) for a direct intro to the bio+health team.</t>
         </is>
       </c>
       <c r="AB3" s="7" t="inlineStr">
@@ -1152,12 +1152,12 @@
       </c>
       <c r="AC3" s="8" t="inlineStr">
         <is>
-          <t>https://a16z.com/infinite-healthcare-whats-it-worth/; https://a16z.com/author/julie-yoo/</t>
+          <t>https://a16z.com/infinite-healthcare-whats-it-worth/; https://www.dlapiper.com/en-us/news/2026/06/dla-piper-advises-andreessen-horowitz-on-usd30-million-investment-in-prosper-ai</t>
         </is>
       </c>
       <c r="AD3" s="8" t="inlineStr">
         <is>
-          <t>Emails inferred/unverified: julie@a16z.com (~55%) or jyoo@a16z.com (~62%).</t>
+          <t>Warm path via DLA Piper counsel (Seidenfeld led an a16z health-AI deal); score contingent on DLA making the intro. Emails inferred/unverified: julie@a16z.com (~55%) or jyoo@a16z.com (~62%).</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
-          <t>LinkedIn or a Lux portfolio founder; no named node confirmed.</t>
+          <t>PLAUSIBLE via DLA Piper: SF partner Jonathan Axelrad represents Lux in financings; intro would hand off from Seidenfeld to Axelrad. Confirm with DLA.</t>
         </is>
       </c>
       <c r="Q5" s="9" t="n">
@@ -1389,14 +1389,14 @@
         <v>0</v>
       </c>
       <c r="U5" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V5" s="9" t="n">
         <v>4</v>
       </c>
       <c r="W5" s="10">
         <f>MAX(0,ROUND(Q5/5*Weights!$B$3+R5/5*Weights!$B$4+S5/5*Weights!$B$5+T5/5*Weights!$B$6+U5/5*Weights!$B$7+V5/5*Weights!$B$8-L5*Weights!$B$9,0))</f>
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="X5" s="10" t="str">
         <f>IF(W5&gt;=Weights!$B$12,"A",IF(W5&gt;=Weights!$B$13,"B","C"))</f>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="AA5" s="8" t="inlineStr">
         <is>
-          <t>Verify a recent Shakir health/AI deal; find intro.</t>
+          <t>Ask DLA (Axelrad) about a Lux intro to Deena Shakir; verify email.</t>
         </is>
       </c>
       <c r="AB5" s="7" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="AC5" s="8" t="inlineStr">
         <is>
-          <t>https://www.luxcapital.com/people; https://www.linkedin.com/in/deenashakir</t>
+          <t>https://www.luxcapital.com/people; https://www.dlapiper.com/en/people/a/jonathan-axelrad</t>
         </is>
       </c>
       <c r="AD5" s="8" t="inlineStr">
         <is>
-          <t>Adam Goulburn is at Dimension, NOT Lux. Email inferred/unverified: deena.shakir@luxcapital.com (pattern first.last ~90%).</t>
+          <t>Adam Goulburn is at Dimension, NOT Lux. Warm path via DLA partner Axelrad (represents Lux); contingent on the hand-off. Email inferred/unverified: deena.shakir@luxcapital.com (pattern first.last ~90%).</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Kraus co-hosts healthcare content; engagement warm-up. No named node.</t>
+          <t>PLAUSIBLE via DLA Piper: Bessemer is a named DLA VC investor-client (repeat deal counsel). Ask which DLA partner currently covers the BVP relationship.</t>
         </is>
       </c>
       <c r="Q16" s="9" t="n">
@@ -2885,14 +2885,14 @@
         <v>0</v>
       </c>
       <c r="U16" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V16" s="9" t="n">
         <v>4</v>
       </c>
       <c r="W16" s="10">
         <f>MAX(0,ROUND(Q16/5*Weights!$B$3+R16/5*Weights!$B$4+S16/5*Weights!$B$5+T16/5*Weights!$B$6+U16/5*Weights!$B$7+V16/5*Weights!$B$8-L16*Weights!$B$9,0))</f>
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="X16" s="10" t="str">
         <f>IF(W16&gt;=Weights!$B$12,"A",IF(W16&gt;=Weights!$B$13,"B","C"))</f>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="AA16" s="8" t="inlineStr">
         <is>
-          <t>Verify email; confirm seed appetite (BVP leans later).</t>
+          <t>Ask DLA which partner covers Bessemer; confirm seed appetite (BVP leans later).</t>
         </is>
       </c>
       <c r="AB16" s="7" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>Cold with an open inbound process; no named node.</t>
+          <t>PLAUSIBLE via DLA Piper: Basis Set GC Jennifer Lee is a DLA alum (ex-CVC co-chair); a DLA partner who overlapped with her can make a peer intro. Confirm with DLA.</t>
         </is>
       </c>
       <c r="Q20" s="9" t="n">
@@ -3429,14 +3429,14 @@
         <v>3</v>
       </c>
       <c r="U20" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V20" s="9" t="n">
         <v>5</v>
       </c>
       <c r="W20" s="10">
         <f>MAX(0,ROUND(Q20/5*Weights!$B$3+R20/5*Weights!$B$4+S20/5*Weights!$B$5+T20/5*Weights!$B$6+U20/5*Weights!$B$7+V20/5*Weights!$B$8-L20*Weights!$B$9,0))</f>
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="X20" s="10" t="str">
         <f>IF(W20&gt;=Weights!$B$12,"A",IF(W20&gt;=Weights!$B$13,"B","C"))</f>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AA20" s="8" t="inlineStr">
         <is>
-          <t>Lead with iViz (AI data workbench); confirm basisset.com vs basisset.ventures domain before emailing.</t>
+          <t>Ask DLA about an alumni intro to GC Jennifer Lee / partner Lan Xuezhao; lead with iViz.</t>
         </is>
       </c>
       <c r="AB20" s="7" t="inlineStr">
@@ -3464,12 +3464,12 @@
       </c>
       <c r="AC20" s="8" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Basis_Set_Ventures; https://www.basisset.com/portfolio</t>
+          <t>https://en.wikipedia.org/wiki/Basis_Set_Ventures; https://www.basisset.com/basis-set-faq</t>
         </is>
       </c>
       <c r="AD20" s="8" t="inlineStr">
         <is>
-          <t>Verified. Email lan@basisset.com is Verified (pattern firstname@basisset.com); some databases list basisset.ventures, confirm first. $2-3M seed check fits as co-lead/participant more than a full seed lead.</t>
+          <t>Verified. Warm path via DLA alumni tie to GC Jennifer Lee; contingent on DLA making it. Email lan@basisset.com is Verified (pattern firstname@basisset.com); some databases list basisset.ventures, confirm first. $2-3M seed check fits as co-lead/participant more than a full seed lead.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-target for infrastructure pivot + $6M seed; add intro-list PDF
Reflects the Oct 2026 deck's change in company approach (drug-development
infrastructure / system of record, with Foresight Base the program record;
modules switch on by stage). Adds a third investor door (enterprise /
vertical-SaaS / dev-infrastructure) and corrects the round to a $6M seed.

- Workbook: updated round context to the infrastructure positioning and
  $6M seed; re-scored check against a $6M seed lead (Conviction 4->5,
  Obvious 3->5), lifting both into Tier A (now 11 Tier A); added infra-fit
  notes for Bessemer and 8VC.
- dla-intro-list.md: new infrastructure one-liner; validation stated as
  retrospective with NSCLC in PoC.
- techbio-vc-targets.md: positioning-update callout.
- Added coharts-investor-intro-list.pdf (brand-styled, forwardable).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AASgEHUdi3Eu3cEx97KCR
</commit_message>
<xml_diff>
--- a/fundraising/coharts-seed-investor-pipeline.xlsx
+++ b/fundraising/coharts-seed-investor-pipeline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Pipeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weights" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline'!$A$1:$AD$31</definedName>
@@ -555,7 +555,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Institutional Seed; target pre-money $25M to $35M (confirm target raise and lead vs participant). Coharts: An Applied AI company, IaaS (never SaaS). Two products: iViz (AI data-analysis workbench, self-serve/PLG) and Foresight (clinical trial simulation, Simulate Success Before Patient One). Traction/proof: Tempus proof-of-concept partnership; Synthon pilot; Foresight validated against real clinical trials both retrospectively and prospectively (including LEAP and TDM1). Angel round closed Aug 2026 on a legacy pre-money SAFE at a $17.5M cap. Most check sizes are Unknown pending PitchBook; personal emails are inferred unless marked Verified. None of these firms are in the HubSpot pipeline (CRM holds pharma/CRO/biotech BD accounts, not investors). CONFLICT FLAGGED: Radical Ventures holds Unlearn.AI (direct Foresight competitor). WARM-PATH NODES: (1) Josh Seidenfeld, DLA Piper partner (ex-Cooley Digital Health chair) = legal-partner intros; bumps applied to a16z (strong), Bessemer, Lux, Basis Set (plausible), all CONTINGENT on DLA making the intro. (2) Johnny (BD, life-sciences venture-banking/investor network) = a separate channel for health/life-sciences investor intros and venture debt later; NOT yet scored, pending named funds he can open. Other firms remain warm-path 1-2 pending named nodes.</t>
+          <t>Institutional Seed, $6M target (valuation TBD with lead; ~26 months runway). POSITIONING UPDATE per Oct 2026 deck: Coharts = drug-development INFRASTRUCTURE, 'one record per program, from first assay to filing, with the models built in.' Foresight Base is the program record ($2K/program/month; Part 11 + ICH E6(R3) data management) with modules (PRISM, ATHENA, BEAM, CTS, iViz) switching on by stage. Applied AI, IaaS (never SaaS). Now also competes with the record/eTMF vaults (Veeva, Medidata Rave, Benchling), not only simulation tools, adding a THIRD investor door: enterprise / vertical-SaaS / dev-infrastructure. Validation is RETROSPECTIVE (LEAP Phase 2, bioavailability, failures re-run); NSCLC in PoC. Traction: Tempus POC (results for JPM Jan 2027), Synthon generics pilot complete (paid conversion $250K-$415K), PRISM with 2 pediatric hospitals (FDA grant filed/pending). A $6M seed favors seed-LEADING funds; most check sizes Unknown pending PitchBook; personal emails inferred unless marked Verified. None of these firms are in the HubSpot pipeline. CONFLICT FLAGGED: Radical Ventures holds Unlearn.AI (direct competitor). WARM-PATH NODES: Josh Seidenfeld (DLA Piper) = legal-partner intros (bumps on a16z/Lux/Basis Set/Bessemer, contingent on DLA); Johnny = BD / life-sciences venture-banking contact coordinating the intros. Other firms remain warm-path 1-2 pending named nodes.</t>
         </is>
       </c>
     </row>
@@ -988,11 +988,11 @@
       </c>
       <c r="W2" s="10">
         <f>MAX(0,ROUND(Q2/5*Weights!$B$3+R2/5*Weights!$B$4+S2/5*Weights!$B$5+T2/5*Weights!$B$6+U2/5*Weights!$B$7+V2/5*Weights!$B$8-L2*Weights!$B$9,0))</f>
-        <v>84</v>
-      </c>
-      <c r="X2" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X2" s="10">
         <f>IF(W2&gt;=Weights!$B$12,"A",IF(W2&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y2" s="11" t="inlineStr">
         <is>
@@ -1124,11 +1124,11 @@
       </c>
       <c r="W3" s="10">
         <f>MAX(0,ROUND(Q3/5*Weights!$B$3+R3/5*Weights!$B$4+S3/5*Weights!$B$5+T3/5*Weights!$B$6+U3/5*Weights!$B$7+V3/5*Weights!$B$8-L3*Weights!$B$9,0))</f>
-        <v>84</v>
-      </c>
-      <c r="X3" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X3" s="10">
         <f>IF(W3&gt;=Weights!$B$12,"A",IF(W3&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y3" s="11" t="inlineStr">
         <is>
@@ -1260,11 +1260,11 @@
       </c>
       <c r="W4" s="10">
         <f>MAX(0,ROUND(Q4/5*Weights!$B$3+R4/5*Weights!$B$4+S4/5*Weights!$B$5+T4/5*Weights!$B$6+U4/5*Weights!$B$7+V4/5*Weights!$B$8-L4*Weights!$B$9,0))</f>
-        <v>74</v>
-      </c>
-      <c r="X4" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X4" s="10">
         <f>IF(W4&gt;=Weights!$B$12,"A",IF(W4&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y4" s="11" t="inlineStr">
         <is>
@@ -1396,11 +1396,11 @@
       </c>
       <c r="W5" s="10">
         <f>MAX(0,ROUND(Q5/5*Weights!$B$3+R5/5*Weights!$B$4+S5/5*Weights!$B$5+T5/5*Weights!$B$6+U5/5*Weights!$B$7+V5/5*Weights!$B$8-L5*Weights!$B$9,0))</f>
-        <v>80</v>
-      </c>
-      <c r="X5" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X5" s="10">
         <f>IF(W5&gt;=Weights!$B$12,"A",IF(W5&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y5" s="11" t="inlineStr">
         <is>
@@ -1532,11 +1532,11 @@
       </c>
       <c r="W6" s="10">
         <f>MAX(0,ROUND(Q6/5*Weights!$B$3+R6/5*Weights!$B$4+S6/5*Weights!$B$5+T6/5*Weights!$B$6+U6/5*Weights!$B$7+V6/5*Weights!$B$8-L6*Weights!$B$9,0))</f>
-        <v>72</v>
-      </c>
-      <c r="X6" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X6" s="10">
         <f>IF(W6&gt;=Weights!$B$12,"A",IF(W6&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y6" s="11" t="inlineStr">
         <is>
@@ -1668,11 +1668,11 @@
       </c>
       <c r="W7" s="10">
         <f>MAX(0,ROUND(Q7/5*Weights!$B$3+R7/5*Weights!$B$4+S7/5*Weights!$B$5+T7/5*Weights!$B$6+U7/5*Weights!$B$7+V7/5*Weights!$B$8-L7*Weights!$B$9,0))</f>
-        <v>72</v>
-      </c>
-      <c r="X7" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X7" s="10">
         <f>IF(W7&gt;=Weights!$B$12,"A",IF(W7&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y7" s="11" t="inlineStr">
         <is>
@@ -1804,11 +1804,11 @@
       </c>
       <c r="W8" s="10">
         <f>MAX(0,ROUND(Q8/5*Weights!$B$3+R8/5*Weights!$B$4+S8/5*Weights!$B$5+T8/5*Weights!$B$6+U8/5*Weights!$B$7+V8/5*Weights!$B$8-L8*Weights!$B$9,0))</f>
-        <v>70</v>
-      </c>
-      <c r="X8" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X8" s="10">
         <f>IF(W8&gt;=Weights!$B$12,"A",IF(W8&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y8" s="11" t="inlineStr">
         <is>
@@ -1940,11 +1940,11 @@
       </c>
       <c r="W9" s="10">
         <f>MAX(0,ROUND(Q9/5*Weights!$B$3+R9/5*Weights!$B$4+S9/5*Weights!$B$5+T9/5*Weights!$B$6+U9/5*Weights!$B$7+V9/5*Weights!$B$8-L9*Weights!$B$9,0))</f>
-        <v>68</v>
-      </c>
-      <c r="X9" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X9" s="10">
         <f>IF(W9&gt;=Weights!$B$12,"A",IF(W9&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y9" s="11" t="inlineStr">
         <is>
@@ -2076,11 +2076,11 @@
       </c>
       <c r="W10" s="10">
         <f>MAX(0,ROUND(Q10/5*Weights!$B$3+R10/5*Weights!$B$4+S10/5*Weights!$B$5+T10/5*Weights!$B$6+U10/5*Weights!$B$7+V10/5*Weights!$B$8-L10*Weights!$B$9,0))</f>
-        <v>64</v>
-      </c>
-      <c r="X10" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X10" s="10">
         <f>IF(W10&gt;=Weights!$B$12,"A",IF(W10&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y10" s="11" t="inlineStr">
         <is>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="AD10" s="8" t="inlineStr">
         <is>
-          <t>Email inferred/unverified: kimmy@8vc.com (~76%). For enterprise clinical-data, 8VC bio team may co-fit.</t>
+          <t>Infra fit strengthens: enterprise health-data infrastructure / system-of-record is squarely 8VC's lane. Email inferred/unverified: kimmy@8vc.com (~76%). For enterprise clinical-data, 8VC bio team may co-fit.</t>
         </is>
       </c>
     </row>
@@ -2212,11 +2212,11 @@
       </c>
       <c r="W11" s="10">
         <f>MAX(0,ROUND(Q11/5*Weights!$B$3+R11/5*Weights!$B$4+S11/5*Weights!$B$5+T11/5*Weights!$B$6+U11/5*Weights!$B$7+V11/5*Weights!$B$8-L11*Weights!$B$9,0))</f>
-        <v>66</v>
-      </c>
-      <c r="X11" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X11" s="10">
         <f>IF(W11&gt;=Weights!$B$12,"A",IF(W11&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y11" s="11" t="inlineStr">
         <is>
@@ -2348,11 +2348,11 @@
       </c>
       <c r="W12" s="10">
         <f>MAX(0,ROUND(Q12/5*Weights!$B$3+R12/5*Weights!$B$4+S12/5*Weights!$B$5+T12/5*Weights!$B$6+U12/5*Weights!$B$7+V12/5*Weights!$B$8-L12*Weights!$B$9,0))</f>
-        <v>58</v>
-      </c>
-      <c r="X12" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X12" s="10">
         <f>IF(W12&gt;=Weights!$B$12,"A",IF(W12&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y12" s="11" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         <v>4</v>
       </c>
       <c r="T13" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U13" s="9" t="n">
         <v>2</v>
@@ -2484,11 +2484,11 @@
       </c>
       <c r="W13" s="10">
         <f>MAX(0,ROUND(Q13/5*Weights!$B$3+R13/5*Weights!$B$4+S13/5*Weights!$B$5+T13/5*Weights!$B$6+U13/5*Weights!$B$7+V13/5*Weights!$B$8-L13*Weights!$B$9,0))</f>
-        <v>66</v>
-      </c>
-      <c r="X13" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X13" s="10">
         <f>IF(W13&gt;=Weights!$B$12,"A",IF(W13&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y13" s="11" t="inlineStr">
         <is>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="AA13" s="8" t="inlineStr">
         <is>
-          <t>Verify email; confirm health-software recency.</t>
+          <t>Verify email; confirm health-software recency. $5-12M checks lead a $6M seed cleanly.</t>
         </is>
       </c>
       <c r="AB13" s="7" t="inlineStr">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="W14" s="10">
         <f>MAX(0,ROUND(Q14/5*Weights!$B$3+R14/5*Weights!$B$4+S14/5*Weights!$B$5+T14/5*Weights!$B$6+U14/5*Weights!$B$7+V14/5*Weights!$B$8-L14*Weights!$B$9,0))</f>
-        <v>64</v>
-      </c>
-      <c r="X14" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X14" s="10">
         <f>IF(W14&gt;=Weights!$B$12,"A",IF(W14&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y14" s="11" t="inlineStr">
         <is>
@@ -2756,11 +2756,11 @@
       </c>
       <c r="W15" s="10">
         <f>MAX(0,ROUND(Q15/5*Weights!$B$3+R15/5*Weights!$B$4+S15/5*Weights!$B$5+T15/5*Weights!$B$6+U15/5*Weights!$B$7+V15/5*Weights!$B$8-L15*Weights!$B$9,0))</f>
-        <v>64</v>
-      </c>
-      <c r="X15" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X15" s="10">
         <f>IF(W15&gt;=Weights!$B$12,"A",IF(W15&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y15" s="11" t="inlineStr">
         <is>
@@ -2892,11 +2892,11 @@
       </c>
       <c r="W16" s="10">
         <f>MAX(0,ROUND(Q16/5*Weights!$B$3+R16/5*Weights!$B$4+S16/5*Weights!$B$5+T16/5*Weights!$B$6+U16/5*Weights!$B$7+V16/5*Weights!$B$8-L16*Weights!$B$9,0))</f>
-        <v>66</v>
-      </c>
-      <c r="X16" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X16" s="10">
         <f>IF(W16&gt;=Weights!$B$12,"A",IF(W16&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y16" s="11" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="AD16" s="8" t="inlineStr">
         <is>
-          <t>Morgan Cheatham left BVP for Breyer. Email inferred/unverified: steve@bvp.com (pattern first@bvp.com).</t>
+          <t>Infra fit strengthens under the new positioning: system-of-record / vertical-SaaS is core BVP thesis. Morgan Cheatham left BVP for Breyer. Email inferred/unverified: steve@bvp.com (pattern first@bvp.com).</t>
         </is>
       </c>
     </row>
@@ -3028,11 +3028,11 @@
       </c>
       <c r="W17" s="10">
         <f>MAX(0,ROUND(Q17/5*Weights!$B$3+R17/5*Weights!$B$4+S17/5*Weights!$B$5+T17/5*Weights!$B$6+U17/5*Weights!$B$7+V17/5*Weights!$B$8-L17*Weights!$B$9,0))</f>
-        <v>58</v>
-      </c>
-      <c r="X17" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X17" s="10">
         <f>IF(W17&gt;=Weights!$B$12,"A",IF(W17&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y17" s="11" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         <v>5</v>
       </c>
       <c r="T18" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U18" s="9" t="n">
         <v>1</v>
@@ -3164,11 +3164,11 @@
       </c>
       <c r="W18" s="10">
         <f>MAX(0,ROUND(Q18/5*Weights!$B$3+R18/5*Weights!$B$4+S18/5*Weights!$B$5+T18/5*Weights!$B$6+U18/5*Weights!$B$7+V18/5*Weights!$B$8-L18*Weights!$B$9,0))</f>
-        <v>78</v>
-      </c>
-      <c r="X18" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X18" s="10">
         <f>IF(W18&gt;=Weights!$B$12,"A",IF(W18&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y18" s="11" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="AD18" s="8" t="inlineStr">
         <is>
-          <t>Verified. Only functional inbox embed@conviction.com is confirmed; sarah@conviction.com / mike@conviction.com are inferred, LOW confidence. Mike Vernal (ex-Sequoia, PLG/infra) is a strong alt contact for the iViz self-serve angle.</t>
+          <t>Verified. Check 5: $1M-$25M range comfortably leads a $6M seed. Infra angle fits (Vernal = PLG/infra). Only functional inbox embed@conviction.com is confirmed; sarah@conviction.com / mike@conviction.com inferred, LOW confidence.</t>
         </is>
       </c>
     </row>
@@ -3300,11 +3300,11 @@
       </c>
       <c r="W19" s="10">
         <f>MAX(0,ROUND(Q19/5*Weights!$B$3+R19/5*Weights!$B$4+S19/5*Weights!$B$5+T19/5*Weights!$B$6+U19/5*Weights!$B$7+V19/5*Weights!$B$8-L19*Weights!$B$9,0))</f>
-        <v>53</v>
-      </c>
-      <c r="X19" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X19" s="10">
         <f>IF(W19&gt;=Weights!$B$12,"A",IF(W19&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y19" s="11" t="inlineStr">
         <is>
@@ -3436,11 +3436,11 @@
       </c>
       <c r="W20" s="10">
         <f>MAX(0,ROUND(Q20/5*Weights!$B$3+R20/5*Weights!$B$4+S20/5*Weights!$B$5+T20/5*Weights!$B$6+U20/5*Weights!$B$7+V20/5*Weights!$B$8-L20*Weights!$B$9,0))</f>
-        <v>80</v>
-      </c>
-      <c r="X20" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X20" s="10">
         <f>IF(W20&gt;=Weights!$B$12,"A",IF(W20&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y20" s="11" t="inlineStr">
         <is>
@@ -3572,11 +3572,11 @@
       </c>
       <c r="W21" s="10">
         <f>MAX(0,ROUND(Q21/5*Weights!$B$3+R21/5*Weights!$B$4+S21/5*Weights!$B$5+T21/5*Weights!$B$6+U21/5*Weights!$B$7+V21/5*Weights!$B$8-L21*Weights!$B$9,0))</f>
-        <v>44</v>
-      </c>
-      <c r="X21" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X21" s="10">
         <f>IF(W21&gt;=Weights!$B$12,"A",IF(W21&gt;=Weights!$B$13,"B","C"))</f>
-        <v>C</v>
+        <v/>
       </c>
       <c r="Y21" s="11" t="inlineStr">
         <is>
@@ -3708,11 +3708,11 @@
       </c>
       <c r="W22" s="10">
         <f>MAX(0,ROUND(Q22/5*Weights!$B$3+R22/5*Weights!$B$4+S22/5*Weights!$B$5+T22/5*Weights!$B$6+U22/5*Weights!$B$7+V22/5*Weights!$B$8-L22*Weights!$B$9,0))</f>
-        <v>24</v>
-      </c>
-      <c r="X22" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X22" s="10">
         <f>IF(W22&gt;=Weights!$B$12,"A",IF(W22&gt;=Weights!$B$13,"B","C"))</f>
-        <v>C</v>
+        <v/>
       </c>
       <c r="Y22" s="11" t="inlineStr">
         <is>
@@ -3844,11 +3844,11 @@
       </c>
       <c r="W23" s="10">
         <f>MAX(0,ROUND(Q23/5*Weights!$B$3+R23/5*Weights!$B$4+S23/5*Weights!$B$5+T23/5*Weights!$B$6+U23/5*Weights!$B$7+V23/5*Weights!$B$8-L23*Weights!$B$9,0))</f>
-        <v>66</v>
-      </c>
-      <c r="X23" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X23" s="10">
         <f>IF(W23&gt;=Weights!$B$12,"A",IF(W23&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y23" s="11" t="inlineStr">
         <is>
@@ -3980,11 +3980,11 @@
       </c>
       <c r="W24" s="10">
         <f>MAX(0,ROUND(Q24/5*Weights!$B$3+R24/5*Weights!$B$4+S24/5*Weights!$B$5+T24/5*Weights!$B$6+U24/5*Weights!$B$7+V24/5*Weights!$B$8-L24*Weights!$B$9,0))</f>
-        <v>60</v>
-      </c>
-      <c r="X24" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X24" s="10">
         <f>IF(W24&gt;=Weights!$B$12,"A",IF(W24&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y24" s="11" t="inlineStr">
         <is>
@@ -4116,11 +4116,11 @@
       </c>
       <c r="W25" s="10">
         <f>MAX(0,ROUND(Q25/5*Weights!$B$3+R25/5*Weights!$B$4+S25/5*Weights!$B$5+T25/5*Weights!$B$6+U25/5*Weights!$B$7+V25/5*Weights!$B$8-L25*Weights!$B$9,0))</f>
-        <v>60</v>
-      </c>
-      <c r="X25" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X25" s="10">
         <f>IF(W25&gt;=Weights!$B$12,"A",IF(W25&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y25" s="11" t="inlineStr">
         <is>
@@ -4252,11 +4252,11 @@
       </c>
       <c r="W26" s="10">
         <f>MAX(0,ROUND(Q26/5*Weights!$B$3+R26/5*Weights!$B$4+S26/5*Weights!$B$5+T26/5*Weights!$B$6+U26/5*Weights!$B$7+V26/5*Weights!$B$8-L26*Weights!$B$9,0))</f>
-        <v>58</v>
-      </c>
-      <c r="X26" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X26" s="10">
         <f>IF(W26&gt;=Weights!$B$12,"A",IF(W26&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y26" s="11" t="inlineStr">
         <is>
@@ -4388,11 +4388,11 @@
       </c>
       <c r="W27" s="10">
         <f>MAX(0,ROUND(Q27/5*Weights!$B$3+R27/5*Weights!$B$4+S27/5*Weights!$B$5+T27/5*Weights!$B$6+U27/5*Weights!$B$7+V27/5*Weights!$B$8-L27*Weights!$B$9,0))</f>
-        <v>74</v>
-      </c>
-      <c r="X27" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X27" s="10">
         <f>IF(W27&gt;=Weights!$B$12,"A",IF(W27&gt;=Weights!$B$13,"B","C"))</f>
-        <v>A</v>
+        <v/>
       </c>
       <c r="Y27" s="11" t="inlineStr">
         <is>
@@ -4524,11 +4524,11 @@
       </c>
       <c r="W28" s="10">
         <f>MAX(0,ROUND(Q28/5*Weights!$B$3+R28/5*Weights!$B$4+S28/5*Weights!$B$5+T28/5*Weights!$B$6+U28/5*Weights!$B$7+V28/5*Weights!$B$8-L28*Weights!$B$9,0))</f>
-        <v>54</v>
-      </c>
-      <c r="X28" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X28" s="10">
         <f>IF(W28&gt;=Weights!$B$12,"A",IF(W28&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y28" s="11" t="inlineStr">
         <is>
@@ -4660,11 +4660,11 @@
       </c>
       <c r="W29" s="10">
         <f>MAX(0,ROUND(Q29/5*Weights!$B$3+R29/5*Weights!$B$4+S29/5*Weights!$B$5+T29/5*Weights!$B$6+U29/5*Weights!$B$7+V29/5*Weights!$B$8-L29*Weights!$B$9,0))</f>
-        <v>54</v>
-      </c>
-      <c r="X29" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X29" s="10">
         <f>IF(W29&gt;=Weights!$B$12,"A",IF(W29&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y29" s="11" t="inlineStr">
         <is>
@@ -4796,11 +4796,11 @@
       </c>
       <c r="W30" s="10">
         <f>MAX(0,ROUND(Q30/5*Weights!$B$3+R30/5*Weights!$B$4+S30/5*Weights!$B$5+T30/5*Weights!$B$6+U30/5*Weights!$B$7+V30/5*Weights!$B$8-L30*Weights!$B$9,0))</f>
-        <v>52</v>
-      </c>
-      <c r="X30" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X30" s="10">
         <f>IF(W30&gt;=Weights!$B$12,"A",IF(W30&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y30" s="11" t="inlineStr">
         <is>
@@ -4932,11 +4932,11 @@
       </c>
       <c r="W31" s="10">
         <f>MAX(0,ROUND(Q31/5*Weights!$B$3+R31/5*Weights!$B$4+S31/5*Weights!$B$5+T31/5*Weights!$B$6+U31/5*Weights!$B$7+V31/5*Weights!$B$8-L31*Weights!$B$9,0))</f>
-        <v>64</v>
-      </c>
-      <c r="X31" s="10" t="str">
+        <v/>
+      </c>
+      <c r="X31" s="10">
         <f>IF(W31&gt;=Weights!$B$12,"A",IF(W31&gt;=Weights!$B$13,"B","C"))</f>
-        <v>B</v>
+        <v/>
       </c>
       <c r="Y31" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Oncology Ventures, Silversmith, Care Equity to pipeline (56 firms)
- Oncology Ventures: seed-stage cancer-care data/AI fund; Tier A (70) on
  the strength of an existing CONNECTED CRM relationship with MP Ben
  Freeberg (warm-path 5, work directly). Oncology-only mandate + co-invest
  tendency are the fit caveats; email verified via CRM.
- Silversmith Capital: right thesis (healthcare IT / vertical SaaS) but
  growth-stage ($1.7B Fund V, $20-125M checks) -> Tier B (54), flagged as a
  Series B+ name, not a seed lead.
- Care Equity: off-thesis growth/control PE in life-science lab services
  -> Tier C (42); existing CRM contact (Sofia Etlin) but wrong structure.
Both Oncology Ventures and Care Equity flagged already-in-pipeline (HubSpot).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AASgEHUdi3Eu3cEx97KCR
</commit_message>
<xml_diff>
--- a/fundraising/coharts-seed-investor-pipeline.xlsx
+++ b/fundraising/coharts-seed-investor-pipeline.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline'!$A$1:$AD$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline'!$A$1:$AD$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -543,7 +543,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>56</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD54"/>
+  <dimension ref="A1:AD57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8097,9 +8097,417 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>Oncology Ventures</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Seed-stage cancer-care data/AI fund (single-GP)</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Fund I, $30M (~2024); a ~$62M 2026 figure is unconfirmed</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Pre-seed/seed cancer-care data &amp; tech; often co-invests</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Selective (co-invests often)</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Yes (CRM: lead, CONNECTED)</t>
+        </is>
+      </c>
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>Oncology-only, NON-drug: cancer-care data, AI, interoperability. Strategic LPs Cardinal Health, City of Hope, Moffitt. Does NOT fund therapeutics/devices.</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="inlineStr">
+        <is>
+          <t>Cancer data + AI thesis; Risa/RISA Labs (AI oncology workflow, Apr 2025), Tono, Lumonus, mPATH.</t>
+        </is>
+      </c>
+      <c r="K55" s="8" t="inlineStr">
+        <is>
+          <t>IgniteData / Archer (EHR-to-EDC clinical-trial data transfer) is a soft adjacency to Foresight's data management, not a hard conflict.</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N55" s="7" t="inlineStr">
+        <is>
+          <t>Ben Freeberg</t>
+        </is>
+      </c>
+      <c r="O55" s="7" t="inlineStr">
+        <is>
+          <t>Founder &amp; Managing Partner</t>
+        </is>
+      </c>
+      <c r="P55" s="8" t="inlineStr">
+        <is>
+          <t>DIRECT: existing CONNECTED relationship in the CRM with the MP (last contacted Jun 2026). Work directly, not via DLA.</t>
+        </is>
+      </c>
+      <c r="Q55" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R55" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S55" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="T55" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U55" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="V55" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="W55" s="10">
+        <f>MAX(0,ROUND(Q55/5*Weights!$B$3+R55/5*Weights!$B$4+S55/5*Weights!$B$5+T55/5*Weights!$B$6+U55/5*Weights!$B$7+V55/5*Weights!$B$8-L55*Weights!$B$9,0))</f>
+        <v>70</v>
+      </c>
+      <c r="X55" s="10" t="str">
+        <f>IF(W55&gt;=Weights!$B$12,"A",IF(W55&gt;=Weights!$B$13,"B","C"))</f>
+        <v>A</v>
+      </c>
+      <c r="Y55" s="11" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="Z55" s="7" t="inlineStr">
+        <is>
+          <t>Nate</t>
+        </is>
+      </c>
+      <c r="AA55" s="8" t="inlineStr">
+        <is>
+          <t>Work the existing Ben Freeberg relationship directly; front an oncology-program angle. Note co-invest tendency (line up a lead).</t>
+        </is>
+      </c>
+      <c r="AB55" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="AC55" s="8" t="inlineStr">
+        <is>
+          <t>https://www.hcinnovationgroup.com/finance-revenue-cycle/news/55136523/oncology-focused-venture-capital-firm-closes-30m-fund; https://www.crunchbase.com/organization/oncology-ventures</t>
+        </is>
+      </c>
+      <c r="AD55" s="8" t="inlineStr">
+        <is>
+          <t>Already in HubSpot (lead, CONNECTED). Email ben@oncology.ventures VERIFIED via CRM contact. Warm-path 5 = direct existing relationship. Oncology-only mandate is the main fit caveat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Silversmith Capital Partners</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Growth-equity firm (healthcare IT / vertical SaaS)</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Fund V, $1.7B, closed Jul 2025 ($5B+ AUM)</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Growth-stage (Series B+); minority or majority</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>$20M to $125M</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>No (growth-stage)</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I56" s="8" t="inlineStr">
+        <is>
+          <t>Deep Healthcare IT &amp; Services book: Iodine Software (clinical AI/CDI), Panalgo (RWD/HEOR), Centauri, LifeStance, Nordic.</t>
+        </is>
+      </c>
+      <c r="J56" s="8" t="inlineStr">
+        <is>
+          <t>Vertical SaaS + information services; some AI (Iodine clinical AI). Not an AI-for-science specialist.</t>
+        </is>
+      </c>
+      <c r="K56" s="8" t="inlineStr">
+        <is>
+          <t>Panalgo (RWD/HEOR analytics) is adjacent to iViz but exited to Norstella (no longer active); not a live conflict.</t>
+        </is>
+      </c>
+      <c r="L56" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N56" s="7" t="inlineStr">
+        <is>
+          <t>Jeff Crisan</t>
+        </is>
+      </c>
+      <c r="O56" s="7" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Managing Partner, Healthcare IT &amp; Services (alt: Jim Quagliaroli)</t>
+        </is>
+      </c>
+      <c r="P56" s="8" t="inlineStr">
+        <is>
+          <t>Cold; no named node.</t>
+        </is>
+      </c>
+      <c r="Q56" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="R56" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="S56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="T56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="U56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V56" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="W56" s="10">
+        <f>MAX(0,ROUND(Q56/5*Weights!$B$3+R56/5*Weights!$B$4+S56/5*Weights!$B$5+T56/5*Weights!$B$6+U56/5*Weights!$B$7+V56/5*Weights!$B$8-L56*Weights!$B$9,0))</f>
+        <v>54</v>
+      </c>
+      <c r="X56" s="10" t="str">
+        <f>IF(W56&gt;=Weights!$B$12,"A",IF(W56&gt;=Weights!$B$13,"B","C"))</f>
+        <v>B</v>
+      </c>
+      <c r="Y56" s="11" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="Z56" s="7" t="inlineStr">
+        <is>
+          <t>Nate</t>
+        </is>
+      </c>
+      <c r="AA56" s="8" t="inlineStr">
+        <is>
+          <t>WRONG STAGE for a $6M seed ($20M+ checks). File for Series B+; keep Jeff Crisan warm.</t>
+        </is>
+      </c>
+      <c r="AB56" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="AC56" s="8" t="inlineStr">
+        <is>
+          <t>https://www.silversmith.com/news/silversmith-capital-partners-closes-1-7-billion-fifth-fund; https://www.silversmith.com/portfolio</t>
+        </is>
+      </c>
+      <c r="AD56" s="8" t="inlineStr">
+        <is>
+          <t>Right thesis (Door C, healthcare IT / vertical SaaS), wrong stage. Score 54 overstates seed-fit; treat as a later-round name. Email jcrisan@silversmith.com inferred (ZoomInfo j***@silversmith.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Care Equity</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Private equity (growth/control, life-science tools &amp; services)</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Care Equity II, $302M (Oct 2022); Fund I $125M (~$425M AUM)</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Growth/buyout PE; NOT venture seed</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Unknown (8-figure PE checks)</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Yes (CRM: lead)</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
+          <t>Wet-lab / bioanalytics tools &amp; services: OmicScouts (proteomics, exited to Momentum Mar 2025), TATAA Biocenter, Sapient Bioanalytics.</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="inlineStr">
+        <is>
+          <t>None found; no AI/software-infrastructure holdings.</t>
+        </is>
+      </c>
+      <c r="K57" s="8" t="inlineStr">
+        <is>
+          <t>None competing with Foresight/iViz; portfolio is lab services.</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N57" s="7" t="inlineStr">
+        <is>
+          <t>Sofia Etlin (firm: Peter Batesko, Founder/CEO)</t>
+        </is>
+      </c>
+      <c r="O57" s="7" t="inlineStr">
+        <is>
+          <t>CRM contact</t>
+        </is>
+      </c>
+      <c r="P57" s="8" t="inlineStr">
+        <is>
+          <t>Existing CRM contact (Sofia Etlin, lead stage); lighter than Oncology Ventures. Work directly if pursued.</t>
+        </is>
+      </c>
+      <c r="Q57" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R57" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S57" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="T57" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="U57" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="V57" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="W57" s="10">
+        <f>MAX(0,ROUND(Q57/5*Weights!$B$3+R57/5*Weights!$B$4+S57/5*Weights!$B$5+T57/5*Weights!$B$6+U57/5*Weights!$B$7+V57/5*Weights!$B$8-L57*Weights!$B$9,0))</f>
+        <v>42</v>
+      </c>
+      <c r="X57" s="10" t="str">
+        <f>IF(W57&gt;=Weights!$B$12,"A",IF(W57&gt;=Weights!$B$13,"B","C"))</f>
+        <v>C</v>
+      </c>
+      <c r="Y57" s="11" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="Z57" s="7" t="inlineStr">
+        <is>
+          <t>Nate</t>
+        </is>
+      </c>
+      <c r="AA57" s="8" t="inlineStr">
+        <is>
+          <t>PASS: off-thesis PE (control in lab tools/services), wrong structure for a $6M software seed.</t>
+        </is>
+      </c>
+      <c r="AB57" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="AC57" s="8" t="inlineStr">
+        <is>
+          <t>https://pitchbook.com/profiles/investor/458093-80; https://www.privateequityinternational.com/institution-profiles/care-equity.html</t>
+        </is>
+      </c>
+      <c r="AD57" s="8" t="inlineStr">
+        <is>
+          <t>Already in HubSpot (lead). Email sofia@careequity.com VERIFIED via CRM; firm head Peter Batesko (peter@careequity.com inferred). Off-thesis growth/control PE in life-science lab services.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AD54"/>
-  <conditionalFormatting sqref="W2:W54">
+  <autoFilter ref="A1:AD57"/>
+  <conditionalFormatting sqref="W2:W57">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -8112,14 +8520,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="Y2:Y254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Researching,Intro requested,Intro made,First meeting,Diligence,Term sheet,Closed,Passed"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q254 R2:R254 S2:S254 T2:T254 U2:U254 V2:V254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="Q2:Q257 R2:R257 S2:S257 T2:T257 U2:U257 V2:V257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="L2:L254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="L2:L257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -8320,7 +8728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9923,6 +10331,141 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>Oncology Ventures</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>$30M cancer-focused seed fund; non-drug mandate</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>HC Innovation Group</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>https://www.hcinnovationgroup.com/finance-revenue-cycle/news/55136523/oncology-focused-venture-capital-firm-closes-30m-fund</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Oncology Ventures</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>Ben Freeberg MP, CONNECTED contact</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>HubSpot CRM</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>HubSpot company 330285638360 / contact 508812255971</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Silversmith Capital Partners</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>Fund V $1.7B Jul 2025; $20-125M checks; healthcare-IT book</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Silversmith</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>https://www.silversmith.com/news/silversmith-capital-partners-closes-1-7-billion-fifth-fund</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Care Equity</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Care Equity II $302M Oct 2022; life-science PE</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>PitchBook</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>https://pitchbook.com/profiles/investor/458093-80</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Care Equity</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Sofia Etlin CRM contact</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>HubSpot CRM</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>HubSpot company 348445133500 / contact 558213895894</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NFX (Tier A, top) and Pioneer Fund to pipeline (58 firms)
- NFX: thesis-perfect seed lead (Fund IV $325M, NFX Bio + core AI-infra
  thesis) with an ACTIVE product review since Jan 2026 -> warm-path 5,
  status First meeting, fit 98 (top of pipeline). Work directly, not via
  DLA; Omri Amirav-Drory (NFX Bio) is the bridge, core fund (Currier) the
  alt for the software-infra profile. No conflicts.
- Pioneer Fund: YC-alumni co-investment fund (not Daniel Gross's Pioneer).
  Founder knows Dave (likely Dave Messina, GP) -> warm-path 4, Tier B (56).
  Does not lead, small checks, YC gate -> worth a conversation, not a lead.
Neither in the CRM.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AASgEHUdi3Eu3cEx97KCR
</commit_message>
<xml_diff>
--- a/fundraising/coharts-seed-investor-pipeline.xlsx
+++ b/fundraising/coharts-seed-investor-pipeline.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline'!$A$1:$AD$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipeline'!$A$1:$AD$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -543,7 +543,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>58</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD57"/>
+  <dimension ref="A1:AD59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8505,9 +8505,281 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>NFX</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Pre-seed/seed VC (network effects; NFX Bio practice)</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco, CA / Herzliya</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Fund IV, $325M, closed end 2024 (~$1.5B AUM)</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Pre-seed and seed; leads</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>~$1.5M to $5M initial (avg $4-5M, Fund IV)</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>No (active review since Jan 2026)</t>
+        </is>
+      </c>
+      <c r="I58" s="8" t="inlineStr">
+        <is>
+          <t>NFX Bio (TechBio/AI-x-bio): led ImmuneBridge $8M seed (Mar 2026), co-led Cyclana Bio (Oct 2025), Mana.bio (Sep 2025), Mammoth Biosciences, C2i Genomics. IC incl. Emily Leproust (Twist CEO).</t>
+        </is>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
+          <t>Core NFX thesis funds AI infrastructure, data tooling, developer platforms, and vertical AI (published thesis + portfolio).</t>
+        </is>
+      </c>
+      <c r="K58" s="8" t="inlineStr">
+        <is>
+          <t>NFX Bio holdings are wet-biology (CRISPR, drug delivery, vaccines); no trial-sim / in-silico-outcome company. No conflict.</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
+        <is>
+          <t>Omri Amirav-Drory, PhD (alt: James Currier, core fund)</t>
+        </is>
+      </c>
+      <c r="O58" s="7" t="inlineStr">
+        <is>
+          <t>General Partner &amp; Head of NFX Bio</t>
+        </is>
+      </c>
+      <c r="P58" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE: NFX has been reviewing Coharts' product since Jan 2026 (in-flight relationship). Work directly, not via DLA.</t>
+        </is>
+      </c>
+      <c r="Q58" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="R58" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="S58" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="T58" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="U58" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="V58" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="W58" s="10">
+        <f>MAX(0,ROUND(Q58/5*Weights!$B$3+R58/5*Weights!$B$4+S58/5*Weights!$B$5+T58/5*Weights!$B$6+U58/5*Weights!$B$7+V58/5*Weights!$B$8-L58*Weights!$B$9,0))</f>
+        <v>98</v>
+      </c>
+      <c r="X58" s="10" t="str">
+        <f>IF(W58&gt;=Weights!$B$12,"A",IF(W58&gt;=Weights!$B$13,"B","C"))</f>
+        <v>A</v>
+      </c>
+      <c r="Y58" s="11" t="inlineStr">
+        <is>
+          <t>First meeting</t>
+        </is>
+      </c>
+      <c r="Z58" s="7" t="inlineStr">
+        <is>
+          <t>Nate</t>
+        </is>
+      </c>
+      <c r="AA58" s="8" t="inlineStr">
+        <is>
+          <t>Drive the existing NFX review to a term sheet. Omri (NFX Bio) is the domain bridge; route the software-infra profile to the core fund (Currier) if Bio stalls on 'wet-lab only'. Confirm where the eval stands.</t>
+        </is>
+      </c>
+      <c r="AB58" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="AC58" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nfx.com/post/nfx-fund-iv; https://www.nfx.com/team/omri-amirav-drory</t>
+        </is>
+      </c>
+      <c r="AD58" s="8" t="inlineStr">
+        <is>
+          <t>TOP PRIORITY: thesis-perfect seed lead + active product review since Jan 2026. Caveat: NFX Bio leans wet-lab bioplatforms, so Coharts' software/regulatory-IaaS profile may fit the core AI-infra fund better. Email omri@nfx.com Inferred (first@nfx.com pattern ~85%). Move status to Diligence/Term sheet as the review advances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Pioneer Fund</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>YC-alumni co-investment fund (sector-agnostic + AI/ML and Bio/Health sleeves)</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Debut fund ~$20M (2018); multiple vehicles since; current flagship size Unknown</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Pre-seed/seed; co-invests alongside YC, does not lead</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>~$150K to $250K avg (some $500K-$2M)</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>No (co-invests)</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I59" s="8" t="inlineStr">
+        <is>
+          <t>Bio+Health sleeve; ~14 therapeutics holdings. Argon AI (pharma AI copilot, $5.5M seed Jul 2025), ParcelBio ($13.2M, 2026), Olio Labs, Ply Health, Resvita Bio.</t>
+        </is>
+      </c>
+      <c r="J59" s="8" t="inlineStr">
+        <is>
+          <t>AI/ML sub-fund; Argon AI (pharma AI) among holdings.</t>
+        </is>
+      </c>
+      <c r="K59" s="8" t="inlineStr">
+        <is>
+          <t>Argon AI (pharma AI clinical/competitive-intelligence copilot) is a mild adjacency to the 'intelligence layer'/iViz, not a CTS/in-silico competitor.</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N59" s="7" t="inlineStr">
+        <is>
+          <t>Dave Messina (GP, Bio+Health) - founder's contact</t>
+        </is>
+      </c>
+      <c r="O59" s="7" t="inlineStr">
+        <is>
+          <t>General Partner (alt: AI Fund GPs Francesco Mosconi / Rajiv Bhat)</t>
+        </is>
+      </c>
+      <c r="P59" s="8" t="inlineStr">
+        <is>
+          <t>Founder knows Dave (likely Dave Messina, GP, Bio+Health). Direct warm node. Work directly.</t>
+        </is>
+      </c>
+      <c r="Q59" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R59" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="S59" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="T59" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="U59" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="V59" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="W59" s="10">
+        <f>MAX(0,ROUND(Q59/5*Weights!$B$3+R59/5*Weights!$B$4+S59/5*Weights!$B$5+T59/5*Weights!$B$6+U59/5*Weights!$B$7+V59/5*Weights!$B$8-L59*Weights!$B$9,0))</f>
+        <v>56</v>
+      </c>
+      <c r="X59" s="10" t="str">
+        <f>IF(W59&gt;=Weights!$B$12,"A",IF(W59&gt;=Weights!$B$13,"B","C"))</f>
+        <v>B</v>
+      </c>
+      <c r="Y59" s="11" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="Z59" s="7" t="inlineStr">
+        <is>
+          <t>Nate</t>
+        </is>
+      </c>
+      <c r="AA59" s="8" t="inlineStr">
+        <is>
+          <t>Use the Dave relationship for a read/signal, but Pioneer co-invests (not a lead), writes small checks, and gates largely to YC companies. Confirm YC eligibility; do not count on it to lead.</t>
+        </is>
+      </c>
+      <c r="AB59" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="AC59" s="8" t="inlineStr">
+        <is>
+          <t>https://www.pioneerfund.vc; https://www.crunchbase.com/organization/pioneer-fund</t>
+        </is>
+      </c>
+      <c r="AD59" s="8" t="inlineStr">
+        <is>
+          <t>YC-alumni fund (pioneerfund.vc), NOT Daniel Gross's Pioneer. Warm via 'Dave' (likely Dave Messina). Non-lead + YC gate + small checks cap the fit; the Dave relationship is why it is worth a conversation. Email pattern Unknown, do not guess.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AD57"/>
-  <conditionalFormatting sqref="W2:W57">
+  <autoFilter ref="A1:AD59"/>
+  <conditionalFormatting sqref="W2:W59">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -8520,14 +8792,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="Y2:Y257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Researching,Intro requested,Intro made,First meeting,Diligence,Term sheet,Closed,Passed"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q257 R2:R257 S2:S257 T2:T257 U2:U257 V2:V257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="Q2:Q259 R2:R259 S2:S259 T2:T259 U2:U259 V2:V259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="L2:L257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="L2:L259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -8728,7 +9000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10466,6 +10738,114 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>NFX</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Fund IV $325M end 2024; leads seed; $1.5-5M checks</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Calcalist / NFX</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nfx.com/post/nfx-fund-iv</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>NFX</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>NFX Bio led ImmuneBridge $8M seed (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nfx.com/post/launching-nfx-bio</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Pioneer Fund</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>YC-alumni co-investment fund; AI/ML + Bio/Health sleeves; does not lead</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Crunchbase / web</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/pioneer-fund</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>Pioneer Fund</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>Argon AI $5.5M seed Jul 2025 (Pioneer + YC)</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/argon-ai</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>